<commit_message>
feat(names): derive name Script instead of overloading Language
</commit_message>
<xml_diff>
--- a/data/rules/postNormalization.xlsx
+++ b/data/rules/postNormalization.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547254E1-F50F-44E9-BC3B-63CA0EB53889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218D8F67-B3E0-422A-B0D8-723ACD0CC64D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="42">
   <si>
     <t>priority</t>
   </si>
@@ -121,12 +121,6 @@
     <t>IF_EMPTY</t>
   </si>
   <si>
-    <t>Names[].Language</t>
-  </si>
-  <si>
-    <t>LANGUAGE</t>
-  </si>
-  <si>
     <t>Countries[].CountryName</t>
   </si>
   <si>
@@ -143,6 +137,15 @@
   </si>
   <si>
     <t>NORMALIZE_NUMBER</t>
+  </si>
+  <si>
+    <t>Names[].Script</t>
+  </si>
+  <si>
+    <t>CANONICAL_SCRIPT</t>
+  </si>
+  <si>
+    <t>SCRIPT</t>
   </si>
 </sst>
 </file>
@@ -222,13 +225,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -544,9 +553,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G999"/>
+  <dimension ref="A1:G1000"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="10.6640625" style="4"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="43.83203125" customWidth="1"/>
     <col min="4" max="4" width="19.58203125" customWidth="1"/>
@@ -555,7 +565,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -578,7 +588,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" t="s">
@@ -601,7 +611,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3">
+      <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" t="s">
@@ -624,7 +634,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4">
+      <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
@@ -647,7 +657,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5">
+      <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" t="s">
@@ -658,7 +668,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6">
+      <c r="A6" s="4">
         <v>10</v>
       </c>
       <c r="B6" t="s">
@@ -675,7 +685,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7">
+      <c r="A7" s="4">
         <v>11</v>
       </c>
       <c r="B7" t="s">
@@ -692,7 +702,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8">
+      <c r="A8" s="4">
         <v>12</v>
       </c>
       <c r="B8" t="s">
@@ -709,7 +719,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9">
+      <c r="A9" s="4">
         <v>13</v>
       </c>
       <c r="B9" t="s">
@@ -726,7 +736,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10">
+      <c r="A10" s="4">
         <v>14</v>
       </c>
       <c r="B10" t="s">
@@ -742,8 +752,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11">
+    <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
         <v>15</v>
       </c>
       <c r="B11" t="s">
@@ -759,73 +769,89 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12">
+    <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
         <v>16</v>
       </c>
       <c r="B12" t="s">
         <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F12" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13">
-        <v>20</v>
+    <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>17</v>
       </c>
       <c r="B13" t="s">
         <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
         <v>32</v>
       </c>
       <c r="E13" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F13" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14">
-        <v>18</v>
+      <c r="A14" s="4">
+        <v>20</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>33</v>
+      </c>
+      <c r="D14" t="s">
+        <v>32</v>
       </c>
       <c r="E14" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15">
+      <c r="A15" s="4">
+        <v>18</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
         <v>100</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="17" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="17" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="18" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="19" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="20" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -1808,6 +1834,7 @@
     <row r="997" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="998" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="999" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="1000" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
feat(dates): resolve approximate flag via generic ENUM_NORMALIZE handler
</commit_message>
<xml_diff>
--- a/data/rules/postNormalization.xlsx
+++ b/data/rules/postNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218D8F67-B3E0-422A-B0D8-723ACD0CC64D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E04E8C9C-6C40-487F-B6E0-624EAB096742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="45">
   <si>
     <t>priority</t>
   </si>
@@ -146,6 +146,15 @@
   </si>
   <si>
     <t>SCRIPT</t>
+  </si>
+  <si>
+    <t>ENUM_NORMALIZE</t>
+  </si>
+  <si>
+    <t>Dates[].IsApproximate</t>
+  </si>
+  <si>
+    <t>true=true|yes=true|1=true|circa=true|approximately=true|approx=true|between=true|estimated=true|false=false|no=false|0=false|exact=false|known=false</t>
   </si>
 </sst>
 </file>
@@ -225,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -238,6 +247,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -553,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:G1001"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="4"/>
@@ -562,6 +577,7 @@
     <col min="4" max="4" width="19.58203125" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="19.9140625" customWidth="1"/>
+    <col min="7" max="7" width="33.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -633,7 +649,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -656,37 +672,39 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="83" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
+      <c r="B5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="6" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
         <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="4">
-        <v>11</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
@@ -695,15 +713,15 @@
         <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
@@ -712,32 +730,32 @@
         <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="4">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
         <v>20</v>
@@ -746,15 +764,15 @@
         <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
         <v>20</v>
@@ -763,110 +781,126 @@
         <v>28</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
         <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="E12" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
         <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E13" t="s">
         <v>39</v>
       </c>
       <c r="F13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D14" t="s">
         <v>32</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F14" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>33</v>
+      </c>
+      <c r="D15" t="s">
+        <v>32</v>
       </c>
       <c r="E15" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F15" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
         <v>100</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="18" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="19" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="20" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="21" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="22" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="23" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="24" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="25" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="26" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="28" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="29" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="30" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="31" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="32" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="18" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="20" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="21" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="22" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="23" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="24" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="25" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="26" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="27" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="28" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="29" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="30" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="31" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="32" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="33" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="34" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="35" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -1835,6 +1869,7 @@
     <row r="998" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="999" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="1000" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="1001" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
feat(PDG-3): strip HTML from canonical text in post-normalization
</commit_message>
<xml_diff>
--- a/data/rules/postNormalization.xlsx
+++ b/data/rules/postNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E04E8C9C-6C40-487F-B6E0-624EAB096742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B2D7CC8-0041-4237-A2C7-D614C4CE6F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="47">
   <si>
     <t>priority</t>
   </si>
@@ -155,6 +155,12 @@
   </si>
   <si>
     <t>true=true|yes=true|1=true|circa=true|approximately=true|approx=true|between=true|estimated=true|false=false|no=false|0=false|exact=false|known=false</t>
+  </si>
+  <si>
+    <t>SANITIZE_HTML</t>
+  </si>
+  <si>
+    <t>additionalInfo[].Value</t>
   </si>
 </sst>
 </file>
@@ -568,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1001"/>
+  <dimension ref="A1:G1003"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="4"/>
@@ -704,41 +710,29 @@
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
         <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="4">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="4">
-        <v>12</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
@@ -747,49 +741,49 @@
         <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F9" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
         <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="4">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
         <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="4">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
         <v>20</v>
@@ -798,109 +792,141 @@
         <v>28</v>
       </c>
       <c r="E12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="4">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
         <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F13" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F14" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F15" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
         <v>20</v>
       </c>
       <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F16" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
         <v>36</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E18" t="s">
         <v>37</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F18" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="4">
+    <row r="19" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
         <v>100</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B19" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="19" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="20" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="21" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="22" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="23" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="24" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="25" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="26" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="27" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="28" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="29" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="30" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="31" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="32" spans="1:2" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="20" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="21" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="22" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="23" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="24" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="25" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="26" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="27" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="28" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="29" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="30" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="31" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="32" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="33" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="34" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="35" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -1870,6 +1896,8 @@
     <row r="999" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="1000" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="1001" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="1002" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="1003" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
feat(PDG-21): onboard GPPB blacklisted entities list
</commit_message>
<xml_diff>
--- a/data/rules/postNormalization.xlsx
+++ b/data/rules/postNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B2D7CC8-0041-4237-A2C7-D614C4CE6F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526A931B-28DD-4020-AD3C-47A6233CCB8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="52">
   <si>
     <t>priority</t>
   </si>
@@ -161,6 +161,21 @@
   </si>
   <si>
     <t>additionalInfo[].Value</t>
+  </si>
+  <si>
+    <t>Measures[].EffectiveDate</t>
+  </si>
+  <si>
+    <t>leaves=EffectiveDate,EndDate</t>
+  </si>
+  <si>
+    <t>DATE_WINDOW_STATUS</t>
+  </si>
+  <si>
+    <t>Measures[].Status</t>
+  </si>
+  <si>
+    <t>hold_type=Category|hold_values=TEMPORARY_REMOVED_BLACKLISTED_ENTITIES|hold_status=Inactive</t>
   </si>
 </sst>
 </file>
@@ -184,7 +199,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -194,6 +209,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFE599"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -240,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -259,6 +280,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -574,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1003"/>
+  <dimension ref="A1:G1005"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="4"/>
@@ -730,43 +758,40 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4">
+    <row r="9" spans="1:7" s="8" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="7">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="7">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
         <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="4">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E10" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="4">
-        <v>12</v>
       </c>
       <c r="B11" t="s">
         <v>20</v>
@@ -775,49 +800,49 @@
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F11" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
         <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F12" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="4">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="4">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
@@ -826,97 +851,129 @@
         <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F14" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="4">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="E15" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F15" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E16" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F16" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
         <v>20</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E17" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F17" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>21</v>
+      </c>
+      <c r="D18" t="s">
+        <v>32</v>
       </c>
       <c r="E18" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
+        <v>20</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
         <v>100</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B21" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="21" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="22" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="22" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="23" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="24" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="25" spans="1:6" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -1898,6 +1955,8 @@
     <row r="1001" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="1002" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="1003" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="1004" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="1005" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>